<commit_message>
Remove API Sync and Last Successful Sync from Dashboard
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41912756-105F-4A27-8F34-D8C9958490B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1404D1A-6A37-4F51-8861-EC61D0DB3E9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="67">
   <si>
     <t>Start Date</t>
   </si>
@@ -215,6 +215,15 @@
   </si>
   <si>
     <t>test plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remove api syncs in dashboard </t>
+  </si>
+  <si>
+    <t xml:space="preserve">when anything buddy uninstall appication send send on mssg at support online or offline </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reporting mssg by mail </t>
   </si>
 </sst>
 </file>
@@ -328,7 +337,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -358,6 +367,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -662,7 +674,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -1336,6 +1348,35 @@
       <c r="A34" s="2">
         <v>46274</v>
       </c>
+      <c r="C34" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="25" x14ac:dyDescent="0.35">
+      <c r="A35" s="2">
+        <v>46274</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>53</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F30" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
Remove/hide the "Application" table/section from the Dashboard. - Remove/hide the "Activity Timeline" table/section from the Dashboard.
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1404D1A-6A37-4F51-8861-EC61D0DB3E9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DC545E6-F268-499A-A4ED-49FA95079CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="81">
   <si>
     <t>Start Date</t>
   </si>
@@ -224,6 +224,48 @@
   </si>
   <si>
     <t xml:space="preserve">Reporting mssg by mail </t>
+  </si>
+  <si>
+    <t xml:space="preserve">iemi  empty send im api  or os_type send to backend </t>
+  </si>
+  <si>
+    <t xml:space="preserve">api login </t>
+  </si>
+  <si>
+    <t xml:space="preserve">idle send in window title show there </t>
+  </si>
+  <si>
+    <t>version log  implement in application</t>
+  </si>
+  <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>Fix Seqrite Email Protection for iHRMS Monitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">email error support </t>
+  </si>
+  <si>
+    <t xml:space="preserve">don’t show tracking application in dashboard </t>
+  </si>
+  <si>
+    <t xml:space="preserve">start time and attandance time , if not punch then show </t>
+  </si>
+  <si>
+    <t xml:space="preserve">user laptop health ,CPU,RAM/ and all </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do the task show the assigned task </t>
+  </si>
+  <si>
+    <t xml:space="preserve">add link to login in hrms </t>
+  </si>
+  <si>
+    <t xml:space="preserve">illegal app alter to backend </t>
+  </si>
+  <si>
+    <t>Dashboard / UI/ API</t>
   </si>
 </sst>
 </file>
@@ -337,7 +379,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -363,13 +405,22 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -674,7 +725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -1320,8 +1371,8 @@
       <c r="E32" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="F32" s="8" t="s">
-        <v>53</v>
+      <c r="F32" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
@@ -1348,6 +1399,9 @@
       <c r="A34" s="2">
         <v>46274</v>
       </c>
+      <c r="B34" s="2">
+        <v>46274</v>
+      </c>
       <c r="C34" s="3" t="s">
         <v>24</v>
       </c>
@@ -1357,14 +1411,17 @@
       <c r="E34" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="F34" s="8" t="s">
-        <v>53</v>
+      <c r="F34" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="25" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>46274</v>
       </c>
+      <c r="B35" s="2">
+        <v>46275</v>
+      </c>
       <c r="C35" s="11" t="s">
         <v>66</v>
       </c>
@@ -1374,7 +1431,189 @@
       <c r="E35" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="F35" s="8" t="s">
+      <c r="F35" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B36" s="2">
+        <v>46274</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B37" s="2">
+        <v>46274</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E37" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B38" s="2">
+        <v>46274</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B39" s="2">
+        <v>46274</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39" t="s">
+        <v>72</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" s="2">
+        <v>46275</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E40" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" s="2">
+        <v>46275</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" s="2">
+        <v>46275</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" s="2">
+        <v>46275</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="F43" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44" s="2">
+        <v>46275</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D44" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E44" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" s="2">
+        <v>46275</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D45" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E45" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="F45" s="8" t="s">
         <v>53</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add system health metrics to activity tracking
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DC545E6-F268-499A-A4ED-49FA95079CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A9819C8-60AD-48B2-A7E5-CFD29F5CF1A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1528,8 +1528,8 @@
       <c r="E40" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="F40" s="8" t="s">
-        <v>53</v>
+      <c r="F40" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
@@ -1562,8 +1562,8 @@
       <c r="E42" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="F42" s="8" t="s">
-        <v>53</v>
+      <c r="F42" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Implement Task API Integration in Dashboard
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A9819C8-60AD-48B2-A7E5-CFD29F5CF1A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE0BB15F-9769-4FFC-B2E3-A40D700B8A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1545,8 +1545,8 @@
       <c r="E41" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="F41" s="8" t="s">
-        <v>53</v>
+      <c r="F41" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
fixing the active /tracking in dashboard
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE0BB15F-9769-4FFC-B2E3-A40D700B8A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{363CFA76-59AE-4B2F-BD18-E7F60BA1CAA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="83">
   <si>
     <t>Start Date</t>
   </si>
@@ -266,6 +266,12 @@
   </si>
   <si>
     <t>Dashboard / UI/ API</t>
+  </si>
+  <si>
+    <t>after restart application re start the fail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">improve and assign task not load in dashborad </t>
   </si>
 </sst>
 </file>
@@ -725,7 +731,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -1519,6 +1525,9 @@
       <c r="A40" s="2">
         <v>46275</v>
       </c>
+      <c r="B40" s="2">
+        <v>46275</v>
+      </c>
       <c r="C40" s="3" t="s">
         <v>80</v>
       </c>
@@ -1536,6 +1545,9 @@
       <c r="A41" s="2">
         <v>46275</v>
       </c>
+      <c r="B41" s="2">
+        <v>46276</v>
+      </c>
       <c r="C41" s="3" t="s">
         <v>80</v>
       </c>
@@ -1553,6 +1565,9 @@
       <c r="A42" s="2">
         <v>46275</v>
       </c>
+      <c r="B42" s="2">
+        <v>46275</v>
+      </c>
       <c r="C42" s="3" t="s">
         <v>80</v>
       </c>
@@ -1570,6 +1585,9 @@
       <c r="A43" s="2">
         <v>46275</v>
       </c>
+      <c r="B43" s="2">
+        <v>46276</v>
+      </c>
       <c r="C43" s="3" t="s">
         <v>80</v>
       </c>
@@ -1579,8 +1597,8 @@
       <c r="E43" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="F43" s="8" t="s">
-        <v>53</v>
+      <c r="F43" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
@@ -1615,6 +1633,40 @@
       </c>
       <c r="F45" s="8" t="s">
         <v>53</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" s="2">
+        <v>46279</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E46" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47" s="2">
+        <v>46279</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixing issue on dashboard
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6164CDFF-6EFC-4F7E-BA55-C4901E8376C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C45A04D8-89E6-4958-B289-E73427B24ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="89">
   <si>
     <t>Start Date</t>
   </si>
@@ -288,6 +288,9 @@
   </si>
   <si>
     <t xml:space="preserve">screenshot not upload in backend /db </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not sending log on backend show device_token / 500 error on api </t>
   </si>
 </sst>
 </file>
@@ -744,7 +747,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -1747,6 +1750,9 @@
       <c r="E50" s="13" t="s">
         <v>86</v>
       </c>
+      <c r="F50" s="8" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
@@ -1766,6 +1772,26 @@
       </c>
       <c r="F51" s="6" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A52" s="2">
+        <v>46281</v>
+      </c>
+      <c r="B52" s="2">
+        <v>46281</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E52" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- Added the existing HRMS/iHRMS logo beside the Welcome text. - Added an HRMS button in the Dashboard header/navigation area.
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C45A04D8-89E6-4958-B289-E73427B24ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE0D5DEC-9784-4622-A72D-EF5EB504C3E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1633,14 +1633,17 @@
       <c r="E44" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="F44" s="8" t="s">
-        <v>53</v>
+      <c r="F44" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>46275</v>
       </c>
+      <c r="B45" s="2">
+        <v>46281</v>
+      </c>
       <c r="C45" s="3" t="s">
         <v>57</v>
       </c>
@@ -1739,7 +1742,7 @@
         <v>46280</v>
       </c>
       <c r="B50" s="2">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>84</v>
@@ -1750,8 +1753,8 @@
       <c r="E50" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="F50" s="8" t="s">
-        <v>53</v>
+      <c r="F50" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
@@ -1790,8 +1793,8 @@
       <c r="E52" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="F52" s="8" t="s">
-        <v>53</v>
+      <c r="F52" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement Attendance Calendar and Leave Balance
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BC39D71-8E01-4933-BAED-5B47D624F62B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{499151C3-B4F8-4553-8385-8A586A75F281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="94">
   <si>
     <t>Start Date</t>
   </si>
@@ -297,6 +297,15 @@
   </si>
   <si>
     <t xml:space="preserve">user laptop health ,CPU,RAM/ and all not syns in bakend </t>
+  </si>
+  <si>
+    <t xml:space="preserve">remove  the weekly timeline </t>
+  </si>
+  <si>
+    <t xml:space="preserve">add attandence mark and leaves balance </t>
+  </si>
+  <si>
+    <t>assign task add timesheet fill</t>
   </si>
 </sst>
 </file>
@@ -753,7 +762,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -1819,6 +1828,9 @@
       <c r="E53" s="13" t="s">
         <v>89</v>
       </c>
+      <c r="F53" s="6" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
@@ -1836,6 +1848,9 @@
       <c r="E54" s="13" t="s">
         <v>48</v>
       </c>
+      <c r="F54" s="6" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
@@ -1852,6 +1867,69 @@
       </c>
       <c r="E55" s="13" t="s">
         <v>90</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A56" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B56" s="2">
+        <v>46283</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D56" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E56" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A57" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B57" s="2">
+        <v>46283</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D57" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E57" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F57" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A58" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B58" s="2">
+        <v>46284</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D58" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E58" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="F58" s="8" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Round System Health values before API submission
- Added rounding for existing numeric System Health values before API submission
- Applied standard mathematical rounding to CPU, RAM, disk and other existing numeric metrics
- Preserved existing System Health payload structure and field names
- Kept numeric values as numbers instead of converting them to strings
- Applied rounding only at the payload preparation stage
- Prevented duplicate rounding by using a single formatting step
- Preserved existing System Health collection, API, authentication and sync logic
- Verified that rounded values are sent to the backend without changing other tracking functionality
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{499151C3-B4F8-4553-8385-8A586A75F281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F089333C-6CF3-4CB8-8BDD-3C29A31838AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="100">
   <si>
     <t>Start Date</t>
   </si>
@@ -306,6 +306,24 @@
   </si>
   <si>
     <t>assign task add timesheet fill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">leaves balance leave type </t>
+  </si>
+  <si>
+    <t xml:space="preserve">in dashboard attandence make calender view and improve more </t>
+  </si>
+  <si>
+    <t>login in HRMS</t>
+  </si>
+  <si>
+    <t>Auto login when user link on dashboard button add there global icon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">system health </t>
+  </si>
+  <si>
+    <t xml:space="preserve">round off thr number or digits syns then </t>
   </si>
 </sst>
 </file>
@@ -419,7 +437,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -459,6 +477,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -762,7 +783,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -1725,7 +1746,7 @@
       <c r="D48" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E48" s="13" t="s">
+      <c r="E48" s="9" t="s">
         <v>83</v>
       </c>
       <c r="F48" s="6" t="s">
@@ -1745,7 +1766,7 @@
       <c r="D49" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E49" s="13" t="s">
+      <c r="E49" s="9" t="s">
         <v>85</v>
       </c>
       <c r="F49" s="6" t="s">
@@ -1765,7 +1786,7 @@
       <c r="D50" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E50" s="13" t="s">
+      <c r="E50" s="9" t="s">
         <v>86</v>
       </c>
       <c r="F50" s="6" t="s">
@@ -1785,7 +1806,7 @@
       <c r="D51" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E51" s="13" t="s">
+      <c r="E51" s="9" t="s">
         <v>87</v>
       </c>
       <c r="F51" s="6" t="s">
@@ -1805,7 +1826,7 @@
       <c r="D52" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E52" s="13" t="s">
+      <c r="E52" s="9" t="s">
         <v>88</v>
       </c>
       <c r="F52" s="6" t="s">
@@ -1825,7 +1846,7 @@
       <c r="D53" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E53" s="13" t="s">
+      <c r="E53" s="9" t="s">
         <v>89</v>
       </c>
       <c r="F53" s="6" t="s">
@@ -1845,7 +1866,7 @@
       <c r="D54" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E54" s="13" t="s">
+      <c r="E54" s="9" t="s">
         <v>48</v>
       </c>
       <c r="F54" s="6" t="s">
@@ -1865,7 +1886,7 @@
       <c r="D55" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E55" s="13" t="s">
+      <c r="E55" s="9" t="s">
         <v>90</v>
       </c>
       <c r="F55" s="6" t="s">
@@ -1885,7 +1906,7 @@
       <c r="D56" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E56" s="13" t="s">
+      <c r="E56" s="9" t="s">
         <v>91</v>
       </c>
       <c r="F56" s="6" t="s">
@@ -1905,7 +1926,7 @@
       <c r="D57" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E57" s="13" t="s">
+      <c r="E57" s="9" t="s">
         <v>92</v>
       </c>
       <c r="F57" s="6" t="s">
@@ -1925,11 +1946,88 @@
       <c r="D58" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E58" s="13" t="s">
+      <c r="E58" s="9" t="s">
         <v>93</v>
       </c>
       <c r="F58" s="8" t="s">
         <v>53</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A59" s="2">
+        <v>46284</v>
+      </c>
+      <c r="B59" s="2">
+        <v>46284</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E59" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="F59" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A60" s="2">
+        <v>46284</v>
+      </c>
+      <c r="B60" s="2">
+        <v>46284</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E60" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A61" s="2">
+        <v>46284</v>
+      </c>
+      <c r="C61" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="D61" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E61" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="F61" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A62" s="2">
+        <v>46284</v>
+      </c>
+      <c r="B62" s="2">
+        <v>46284</v>
+      </c>
+      <c r="C62" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E62" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="F62" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Start/Stop Tracking control and update Dashboard status label
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AB30FB6-84BA-4B87-B1CE-CC1CCBC23C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D39090F-A632-483F-A2C0-6E54E6C5E93F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,12 +19,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Project Tracker'!$A$1:$F$30</definedName>
   </definedNames>
   <calcPr calcId="0" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="107">
   <si>
     <t>Start Date</t>
   </si>
@@ -342,6 +341,9 @@
   </si>
   <si>
     <t xml:space="preserve">leaves balance leave type  not load </t>
+  </si>
+  <si>
+    <t xml:space="preserve">add start and stop button </t>
   </si>
 </sst>
 </file>
@@ -455,7 +457,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -495,9 +497,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -801,7 +800,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -1984,7 +1983,7 @@
       <c r="D59" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E59" s="13" t="s">
+      <c r="E59" s="9" t="s">
         <v>94</v>
       </c>
       <c r="F59" s="6" t="s">
@@ -2004,7 +2003,7 @@
       <c r="D60" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E60" s="13" t="s">
+      <c r="E60" s="9" t="s">
         <v>95</v>
       </c>
       <c r="F60" s="6" t="s">
@@ -2018,13 +2017,13 @@
       <c r="B61" s="2">
         <v>46286</v>
       </c>
-      <c r="C61" s="14" t="s">
+      <c r="C61" s="11" t="s">
         <v>96</v>
       </c>
       <c r="D61" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E61" s="13" t="s">
+      <c r="E61" s="9" t="s">
         <v>97</v>
       </c>
       <c r="F61" s="8" t="s">
@@ -2038,13 +2037,13 @@
       <c r="B62" s="2">
         <v>46284</v>
       </c>
-      <c r="C62" s="14" t="s">
+      <c r="C62" s="11" t="s">
         <v>98</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E62" s="13" t="s">
+      <c r="E62" s="9" t="s">
         <v>99</v>
       </c>
       <c r="F62" s="6" t="s">
@@ -2064,7 +2063,7 @@
       <c r="D63" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E63" s="13" t="s">
+      <c r="E63" s="9" t="s">
         <v>104</v>
       </c>
       <c r="F63" s="8" t="s">
@@ -2084,7 +2083,7 @@
       <c r="D64" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E64" s="13" t="s">
+      <c r="E64" s="9" t="s">
         <v>105</v>
       </c>
       <c r="F64" s="8" t="s">
@@ -2098,16 +2097,36 @@
       <c r="B65" s="2">
         <v>46286</v>
       </c>
-      <c r="C65" s="14" t="s">
+      <c r="C65" s="11" t="s">
         <v>101</v>
       </c>
       <c r="D65" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E65" s="13" t="s">
+      <c r="E65" s="9" t="s">
         <v>102</v>
       </c>
       <c r="F65" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A66" s="2">
+        <v>46287</v>
+      </c>
+      <c r="B66" s="2">
+        <v>46287</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D66" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E66" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="F66" s="8" t="s">
         <v>53</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update api change to app controller api
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6684C4A-4B71-42F1-97BA-CD5E95FC4AE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36EFD8BA-2594-44F3-9125-6A56AAC4B5F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,12 +18,24 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Project Tracker'!$A$1:$F$30</definedName>
   </definedNames>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="111">
   <si>
     <t>Start Date</t>
   </si>
@@ -352,6 +364,12 @@
     <t xml:space="preserve">change Smart workspace activity monitoring 
 To
 Smart workspace productivity monitoring and more too </t>
+  </si>
+  <si>
+    <t>version /API</t>
+  </si>
+  <si>
+    <t>update api change for compare version</t>
   </si>
 </sst>
 </file>
@@ -503,11 +521,11 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -811,7 +829,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -2134,7 +2152,7 @@
       <c r="D66" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E66" s="13" t="s">
+      <c r="E66" s="9" t="s">
         <v>106</v>
       </c>
       <c r="F66" s="6" t="s">
@@ -2151,7 +2169,7 @@
       <c r="D67" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E67" s="13" t="s">
+      <c r="E67" s="9" t="s">
         <v>107</v>
       </c>
       <c r="F67" s="8" t="s">
@@ -2171,10 +2189,30 @@
       <c r="D68" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E68" s="14" t="s">
+      <c r="E68" s="13" t="s">
         <v>108</v>
       </c>
       <c r="F68" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A69" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B69" s="2">
+        <v>46293</v>
+      </c>
+      <c r="C69" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="D69" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E69" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="F69" s="6" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
dashboard improve and fix the "Attendance" section/card immediately
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36EFD8BA-2594-44F3-9125-6A56AAC4B5F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D565BB9-5561-4C44-8AE9-10CDC4BD0EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="115">
   <si>
     <t>Start Date</t>
   </si>
@@ -370,6 +370,18 @@
   </si>
   <si>
     <t>update api change for compare version</t>
+  </si>
+  <si>
+    <t>fix the workflow of sending mail to support ihrms mail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All module test by ai </t>
+  </si>
+  <si>
+    <t xml:space="preserve">All module test by ai make a test cases then build the exe file and attache the report </t>
+  </si>
+  <si>
+    <t xml:space="preserve">attandence card improve </t>
   </si>
 </sst>
 </file>
@@ -483,7 +495,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -526,6 +538,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -829,7 +844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -1495,8 +1510,8 @@
       <c r="E33" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="F33" s="8" t="s">
-        <v>53</v>
+      <c r="F33" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
@@ -2213,6 +2228,66 @@
         <v>110</v>
       </c>
       <c r="F69" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A70" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B70" s="2">
+        <v>46293</v>
+      </c>
+      <c r="C70" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="D70" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E70" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="25" x14ac:dyDescent="0.35">
+      <c r="A71" s="2">
+        <v>46294</v>
+      </c>
+      <c r="B71" s="2">
+        <v>46295</v>
+      </c>
+      <c r="C71" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="D71" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E71" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A72" s="2">
+        <v>46296</v>
+      </c>
+      <c r="B72" s="2">
+        <v>46296</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D72" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E72" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="F72" s="6" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve offline sync failure support reporting
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D565BB9-5561-4C44-8AE9-10CDC4BD0EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20153C5E-D379-40D3-B260-E4151D10376D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,8 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Project Tracker'!$A$1:$F$30</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="122">
   <si>
     <t>Start Date</t>
   </si>
@@ -382,6 +381,27 @@
   </si>
   <si>
     <t xml:space="preserve">attandence card improve </t>
+  </si>
+  <si>
+    <t>attandance api</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not match api status of punching </t>
+  </si>
+  <si>
+    <t xml:space="preserve">leave balance api </t>
+  </si>
+  <si>
+    <t xml:space="preserve">count of leaves not apply </t>
+  </si>
+  <si>
+    <t xml:space="preserve">not open sametimes hang </t>
+  </si>
+  <si>
+    <t xml:space="preserve">offline mention when net is off </t>
+  </si>
+  <si>
+    <t xml:space="preserve">when net is offline so done send mssg api not syns on support mail </t>
   </si>
 </sst>
 </file>
@@ -537,10 +557,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -844,7 +864,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -2224,7 +2244,7 @@
       <c r="D69" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E69" s="14" t="s">
+      <c r="E69" s="9" t="s">
         <v>110</v>
       </c>
       <c r="F69" s="6" t="s">
@@ -2238,13 +2258,13 @@
       <c r="B70" s="2">
         <v>46293</v>
       </c>
-      <c r="C70" s="15" t="s">
+      <c r="C70" s="11" t="s">
         <v>73</v>
       </c>
       <c r="D70" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E70" s="14" t="s">
+      <c r="E70" s="9" t="s">
         <v>111</v>
       </c>
       <c r="F70" s="6" t="s">
@@ -2258,13 +2278,13 @@
       <c r="B71" s="2">
         <v>46295</v>
       </c>
-      <c r="C71" s="15" t="s">
+      <c r="C71" s="11" t="s">
         <v>112</v>
       </c>
       <c r="D71" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E71" s="15" t="s">
+      <c r="E71" s="11" t="s">
         <v>113</v>
       </c>
       <c r="F71" s="6" t="s">
@@ -2284,10 +2304,110 @@
       <c r="D72" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E72" s="14" t="s">
+      <c r="E72" s="9" t="s">
         <v>114</v>
       </c>
       <c r="F72" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A73" s="2">
+        <v>46300</v>
+      </c>
+      <c r="B73" s="2">
+        <v>46300</v>
+      </c>
+      <c r="C73" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E73" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A74" s="2">
+        <v>46300</v>
+      </c>
+      <c r="B74" s="2">
+        <v>46300</v>
+      </c>
+      <c r="C74" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E74" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A75" s="2">
+        <v>46300</v>
+      </c>
+      <c r="B75" s="2">
+        <v>46300</v>
+      </c>
+      <c r="C75" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E75" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A76" s="2">
+        <v>46300</v>
+      </c>
+      <c r="B76" s="2">
+        <v>46300</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E76" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A77" s="2">
+        <v>46300</v>
+      </c>
+      <c r="B77" s="2">
+        <v>46300</v>
+      </c>
+      <c r="C77" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D77" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E77" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="F77" s="6" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
monthly attendance UI improving and leave balance
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20153C5E-D379-40D3-B260-E4151D10376D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E516850-A7A5-4153-B6C2-55DF6DE4CBA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Project Tracker'!$A$1:$F$30</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="135">
   <si>
     <t>Start Date</t>
   </si>
@@ -402,6 +402,46 @@
   </si>
   <si>
     <t xml:space="preserve">when net is offline so done send mssg api not syns on support mail </t>
+  </si>
+  <si>
+    <t>API / Attendance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ix the Workpulse Attendance calendar functionality proper not get data </t>
+  </si>
+  <si>
+    <t>start automatic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">after shutdown then logging </t>
+  </si>
+  <si>
+    <t xml:space="preserve">error api </t>
+  </si>
+  <si>
+    <t>implement error api error also send error address on there</t>
+  </si>
+  <si>
+    <t>fix the error api error test send mail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">error support mail </t>
+  </si>
+  <si>
+    <t>mail send only in production level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attandance UI </t>
+  </si>
+  <si>
+    <t xml:space="preserve">improve attendance ui  </t>
+  </si>
+  <si>
+    <t>leave balance  UI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">leave balance remove card add chart bar and table view remove total 
+leave count </t>
   </si>
 </sst>
 </file>
@@ -557,10 +597,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -864,7 +904,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -2318,13 +2358,13 @@
       <c r="B73" s="2">
         <v>46300</v>
       </c>
-      <c r="C73" s="14" t="s">
+      <c r="C73" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D73" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E73" s="15" t="s">
+      <c r="E73" s="9" t="s">
         <v>116</v>
       </c>
       <c r="F73" s="6" t="s">
@@ -2338,13 +2378,13 @@
       <c r="B74" s="2">
         <v>46300</v>
       </c>
-      <c r="C74" s="14" t="s">
+      <c r="C74" s="11" t="s">
         <v>117</v>
       </c>
       <c r="D74" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E74" s="15" t="s">
+      <c r="E74" s="9" t="s">
         <v>118</v>
       </c>
       <c r="F74" s="6" t="s">
@@ -2358,13 +2398,13 @@
       <c r="B75" s="2">
         <v>46300</v>
       </c>
-      <c r="C75" s="14" t="s">
+      <c r="C75" s="11" t="s">
         <v>61</v>
       </c>
       <c r="D75" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E75" s="15" t="s">
+      <c r="E75" s="9" t="s">
         <v>119</v>
       </c>
       <c r="F75" s="6" t="s">
@@ -2384,7 +2424,7 @@
       <c r="D76" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E76" s="15" t="s">
+      <c r="E76" s="9" t="s">
         <v>120</v>
       </c>
       <c r="F76" s="6" t="s">
@@ -2398,18 +2438,167 @@
       <c r="B77" s="2">
         <v>46300</v>
       </c>
-      <c r="C77" s="14" t="s">
+      <c r="C77" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D77" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E77" s="15" t="s">
+      <c r="E77" s="9" t="s">
         <v>121</v>
       </c>
       <c r="F77" s="6" t="s">
         <v>10</v>
       </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A78" s="2">
+        <v>46301</v>
+      </c>
+      <c r="B78" s="2">
+        <v>46301</v>
+      </c>
+      <c r="C78" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E78" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A79" s="2">
+        <v>46301</v>
+      </c>
+      <c r="B79" s="2">
+        <v>46301</v>
+      </c>
+      <c r="C79" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E79" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A80" s="2">
+        <v>46301</v>
+      </c>
+      <c r="B80" s="2">
+        <v>46301</v>
+      </c>
+      <c r="C80" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="D80" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E80" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="F80" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A81" s="2">
+        <v>46302</v>
+      </c>
+      <c r="B81" s="2">
+        <v>46302</v>
+      </c>
+      <c r="C81" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E81" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="F81" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A82" s="2">
+        <v>46302</v>
+      </c>
+      <c r="B82" s="2">
+        <v>46302</v>
+      </c>
+      <c r="C82" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="D82" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E82" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A83" s="2">
+        <v>46302</v>
+      </c>
+      <c r="B83" s="2">
+        <v>46302</v>
+      </c>
+      <c r="C83" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="D83" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E83" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="F83" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="25" x14ac:dyDescent="0.35">
+      <c r="A84" s="2">
+        <v>46302</v>
+      </c>
+      <c r="B84" s="2">
+        <v>46302</v>
+      </c>
+      <c r="C84" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="D84" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E84" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="F84" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A85" s="2">
+        <v>46302</v>
+      </c>
+      <c r="B85" s="2">
+        <v>46302</v>
+      </c>
+      <c r="C85" s="15"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F30" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
Keep the existing UI styling and attendance functionality unchanged.  Avoid changes to APIs, attendance calculations, and unrelated components.
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E516850-A7A5-4153-B6C2-55DF6DE4CBA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA64EB29-1C57-4368-A22E-22B3E9CECAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="138">
   <si>
     <t>Start Date</t>
   </si>
@@ -442,6 +442,15 @@
   <si>
     <t xml:space="preserve">leave balance remove card add chart bar and table view remove total 
 leave count </t>
+  </si>
+  <si>
+    <t xml:space="preserve">attendance api </t>
+  </si>
+  <si>
+    <t xml:space="preserve">exe warning </t>
+  </si>
+  <si>
+    <t xml:space="preserve">warning issue when install </t>
   </si>
 </sst>
 </file>
@@ -904,7 +913,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -2556,7 +2565,7 @@
         <v>46302</v>
       </c>
       <c r="B83" s="2">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="C83" s="15" t="s">
         <v>131</v>
@@ -2567,8 +2576,8 @@
       <c r="E83" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="F83" s="8" t="s">
-        <v>53</v>
+      <c r="F83" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="84" spans="1:6" ht="25" x14ac:dyDescent="0.35">
@@ -2576,7 +2585,7 @@
         <v>46302</v>
       </c>
       <c r="B84" s="2">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="C84" s="11" t="s">
         <v>133</v>
@@ -2587,18 +2596,49 @@
       <c r="E84" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="F84" s="8" t="s">
-        <v>53</v>
+      <c r="F84" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="B85" s="2">
-        <v>46302</v>
-      </c>
-      <c r="C85" s="15"/>
+        <v>46307</v>
+      </c>
+      <c r="C85" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E85" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="F85" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A86" s="2">
+        <v>46307</v>
+      </c>
+      <c r="B86" s="2">
+        <v>46307</v>
+      </c>
+      <c r="C86" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="D86" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E86" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="F86" s="8" t="s">
+        <v>53</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F30" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
additional api implementation and ui or task table fill time sheet
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA64EB29-1C57-4368-A22E-22B3E9CECAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E95583AB-D56D-4F66-9A54-09B43CFF5E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="148">
   <si>
     <t>Start Date</t>
   </si>
@@ -451,6 +451,36 @@
   </si>
   <si>
     <t xml:space="preserve">warning issue when install </t>
+  </si>
+  <si>
+    <t>Date and Ihrms</t>
+  </si>
+  <si>
+    <t>Date Format and Rename HRMS to iHRMS Throughout the Project</t>
+  </si>
+  <si>
+    <t>Improve dashboard attendance and tracking status UI</t>
+  </si>
+  <si>
+    <t>kra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kra is not get in dashboard </t>
+  </si>
+  <si>
+    <t xml:space="preserve">attandence rate improve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">kra table </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ui of kra task table and the submit </t>
+  </si>
+  <si>
+    <t xml:space="preserve">additional task api </t>
+  </si>
+  <si>
+    <t xml:space="preserve">implement additional  api make there ui in dashboard </t>
   </si>
 </sst>
 </file>
@@ -460,7 +490,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -477,6 +507,11 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -517,7 +552,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -560,11 +595,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF9E9E9E"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -610,6 +654,18 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -913,7 +969,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F92"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -2636,7 +2692,127 @@
       <c r="E86" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="F86" s="8" t="s">
+      <c r="F86" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A87" s="2">
+        <v>46308</v>
+      </c>
+      <c r="B87" s="2">
+        <v>46308</v>
+      </c>
+      <c r="C87" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E87" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="F87" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A88" s="2">
+        <v>46308</v>
+      </c>
+      <c r="B88" s="2">
+        <v>46308</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D88" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E88" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="F88" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A89" s="2">
+        <v>46308</v>
+      </c>
+      <c r="B89" s="2">
+        <v>46308</v>
+      </c>
+      <c r="C89" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="D89" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E89" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="F89" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A90" s="2">
+        <v>46308</v>
+      </c>
+      <c r="B90" s="2">
+        <v>46308</v>
+      </c>
+      <c r="C90" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E90" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="F90" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A91" s="2">
+        <v>46309</v>
+      </c>
+      <c r="B91" s="2">
+        <v>46309</v>
+      </c>
+      <c r="C91" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="D91" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E91" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F91" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A92" s="2">
+        <v>46309</v>
+      </c>
+      <c r="B92" s="2">
+        <v>46309</v>
+      </c>
+      <c r="C92" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="D92" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E92" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="F92" s="8" t="s">
         <v>53</v>
       </c>
     </row>

</xml_diff>

<commit_message>
additional task improve , version pop implementation and log show
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E95583AB-D56D-4F66-9A54-09B43CFF5E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF6AFB1-0FF4-4B90-A720-6E93817573A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="151">
   <si>
     <t>Start Date</t>
   </si>
@@ -481,6 +481,16 @@
   </si>
   <si>
     <t xml:space="preserve">implement additional  api make there ui in dashboard </t>
+  </si>
+  <si>
+    <t>version detail</t>
+  </si>
+  <si>
+    <t>version log  implement in application in pop up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">in version log mention in red and green colour and impovent :,new:,fixed:, 
+yeh format mein ho or drop down mein ek scroll and search option </t>
   </si>
 </sst>
 </file>
@@ -649,16 +659,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -969,7 +979,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -2529,7 +2539,7 @@
       <c r="D78" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E78" s="14" t="s">
+      <c r="E78" s="9" t="s">
         <v>123</v>
       </c>
       <c r="F78" s="6" t="s">
@@ -2543,13 +2553,13 @@
       <c r="B79" s="2">
         <v>46301</v>
       </c>
-      <c r="C79" s="15" t="s">
+      <c r="C79" s="11" t="s">
         <v>124</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E79" s="14" t="s">
+      <c r="E79" s="9" t="s">
         <v>125</v>
       </c>
       <c r="F79" s="6" t="s">
@@ -2563,13 +2573,13 @@
       <c r="B80" s="2">
         <v>46301</v>
       </c>
-      <c r="C80" s="15" t="s">
+      <c r="C80" s="11" t="s">
         <v>126</v>
       </c>
       <c r="D80" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E80" s="14" t="s">
+      <c r="E80" s="9" t="s">
         <v>127</v>
       </c>
       <c r="F80" s="6" t="s">
@@ -2583,13 +2593,13 @@
       <c r="B81" s="2">
         <v>46302</v>
       </c>
-      <c r="C81" s="15" t="s">
+      <c r="C81" s="11" t="s">
         <v>126</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E81" s="14" t="s">
+      <c r="E81" s="9" t="s">
         <v>128</v>
       </c>
       <c r="F81" s="6" t="s">
@@ -2603,13 +2613,13 @@
       <c r="B82" s="2">
         <v>46302</v>
       </c>
-      <c r="C82" s="15" t="s">
+      <c r="C82" s="11" t="s">
         <v>129</v>
       </c>
       <c r="D82" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E82" s="14" t="s">
+      <c r="E82" s="9" t="s">
         <v>130</v>
       </c>
       <c r="F82" s="6" t="s">
@@ -2623,13 +2633,13 @@
       <c r="B83" s="2">
         <v>46303</v>
       </c>
-      <c r="C83" s="15" t="s">
+      <c r="C83" s="11" t="s">
         <v>131</v>
       </c>
       <c r="D83" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E83" s="14" t="s">
+      <c r="E83" s="9" t="s">
         <v>132</v>
       </c>
       <c r="F83" s="6" t="s">
@@ -2649,7 +2659,7 @@
       <c r="D84" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E84" s="14" t="s">
+      <c r="E84" s="9" t="s">
         <v>134</v>
       </c>
       <c r="F84" s="6" t="s">
@@ -2663,13 +2673,13 @@
       <c r="B85" s="2">
         <v>46307</v>
       </c>
-      <c r="C85" s="15" t="s">
+      <c r="C85" s="11" t="s">
         <v>135</v>
       </c>
       <c r="D85" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E85" s="14" t="s">
+      <c r="E85" s="9" t="s">
         <v>123</v>
       </c>
       <c r="F85" s="6" t="s">
@@ -2683,13 +2693,13 @@
       <c r="B86" s="2">
         <v>46307</v>
       </c>
-      <c r="C86" s="15" t="s">
+      <c r="C86" s="11" t="s">
         <v>136</v>
       </c>
       <c r="D86" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E86" s="14" t="s">
+      <c r="E86" s="9" t="s">
         <v>137</v>
       </c>
       <c r="F86" s="6" t="s">
@@ -2703,13 +2713,13 @@
       <c r="B87" s="2">
         <v>46308</v>
       </c>
-      <c r="C87" s="15" t="s">
+      <c r="C87" s="11" t="s">
         <v>138</v>
       </c>
       <c r="D87" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E87" s="14" t="s">
+      <c r="E87" s="9" t="s">
         <v>139</v>
       </c>
       <c r="F87" s="6" t="s">
@@ -2729,7 +2739,7 @@
       <c r="D88" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E88" s="14" t="s">
+      <c r="E88" s="9" t="s">
         <v>140</v>
       </c>
       <c r="F88" s="6" t="s">
@@ -2743,13 +2753,13 @@
       <c r="B89" s="2">
         <v>46308</v>
       </c>
-      <c r="C89" s="15" t="s">
+      <c r="C89" s="11" t="s">
         <v>131</v>
       </c>
       <c r="D89" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E89" s="17" t="s">
+      <c r="E89" s="15" t="s">
         <v>143</v>
       </c>
       <c r="F89" s="6" t="s">
@@ -2763,13 +2773,13 @@
       <c r="B90" s="2">
         <v>46308</v>
       </c>
-      <c r="C90" s="15" t="s">
+      <c r="C90" s="11" t="s">
         <v>141</v>
       </c>
       <c r="D90" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E90" s="16" t="s">
+      <c r="E90" s="14" t="s">
         <v>142</v>
       </c>
       <c r="F90" s="6" t="s">
@@ -2783,17 +2793,17 @@
       <c r="B91" s="2">
         <v>46309</v>
       </c>
-      <c r="C91" s="18" t="s">
+      <c r="C91" s="16" t="s">
         <v>144</v>
       </c>
       <c r="D91" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E91" s="19" t="s">
+      <c r="E91" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="F91" s="8" t="s">
-        <v>53</v>
+      <c r="F91" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.35">
@@ -2803,16 +2813,56 @@
       <c r="B92" s="2">
         <v>46309</v>
       </c>
-      <c r="C92" s="18" t="s">
+      <c r="C92" s="16" t="s">
         <v>146</v>
       </c>
       <c r="D92" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E92" s="19" t="s">
+      <c r="E92" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="F92" s="8" t="s">
+      <c r="F92" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A93" s="2">
+        <v>46309</v>
+      </c>
+      <c r="B93" s="2">
+        <v>46309</v>
+      </c>
+      <c r="C93" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="D93" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E93" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="F93" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A94" s="2">
+        <v>46309</v>
+      </c>
+      <c r="B94" s="2">
+        <v>46309</v>
+      </c>
+      <c r="C94" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="D94" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E94" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="F94" s="8" t="s">
         <v>53</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance Release Summary version selector
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF6AFB1-0FF4-4B90-A720-6E93817573A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA84C203-562A-43CC-9C8C-C627F82DB98E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2842,8 +2842,8 @@
       <c r="E93" s="19" t="s">
         <v>149</v>
       </c>
-      <c r="F93" s="8" t="s">
-        <v>53</v>
+      <c r="F93" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="94" spans="1:6" ht="29" x14ac:dyDescent="0.35">
@@ -2851,7 +2851,7 @@
         <v>46309</v>
       </c>
       <c r="B94" s="2">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="C94" s="18" t="s">
         <v>148</v>
@@ -2862,8 +2862,8 @@
       <c r="E94" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="F94" s="8" t="s">
-        <v>53</v>
+      <c r="F94" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix the punch time and timesheet kra
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA84C203-562A-43CC-9C8C-C627F82DB98E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9151B404-E03C-4FE6-B609-5417B8DAFA24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="152">
   <si>
     <t>Start Date</t>
   </si>
@@ -491,6 +491,9 @@
   <si>
     <t xml:space="preserve">in version log mention in red and green colour and impovent :,new:,fixed:, 
 yeh format mein ho or drop down mein ek scroll and search option </t>
+  </si>
+  <si>
+    <t>additional task submit problem</t>
   </si>
 </sst>
 </file>
@@ -979,7 +982,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -2866,6 +2869,46 @@
         <v>10</v>
       </c>
     </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A95" s="2">
+        <v>46310</v>
+      </c>
+      <c r="B95" s="2">
+        <v>46311</v>
+      </c>
+      <c r="C95" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E95" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="F95" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A96" s="2">
+        <v>46310</v>
+      </c>
+      <c r="B96" s="2">
+        <v>46310</v>
+      </c>
+      <c r="C96" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E96" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="F96" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F30" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Improve app recovery, session persistence, and startup behavior
- Investigate and improve Windows application restart and recovery behavior.
- Improve session restoration to avoid unnecessary repeated login after restart when the existing session remains valid.
- Fix duplicate application instances and single-instance startup handling.
- Investigate automatic company-code prefill on fresh installations.
- Prevent unwanted console windows from appearing during application startup.
- Preserve existing authentication, tracking, synchronization, API contracts, and application functionality.
- Maintain existing logging and error reporting for startup and recovery diagnostics.
- Verify Windows packaging and startup behavior after the changes.
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9151B404-E03C-4FE6-B609-5417B8DAFA24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C14CAABD-AF40-4198-ABA9-9B2FB5B39BFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="158">
   <si>
     <t>Start Date</t>
   </si>
@@ -494,6 +494,24 @@
   </si>
   <si>
     <t>additional task submit problem</t>
+  </si>
+  <si>
+    <t>kra api</t>
+  </si>
+  <si>
+    <t xml:space="preserve">miss match number and data api </t>
+  </si>
+  <si>
+    <t>UI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">circular rounded card same format in all project or tab is not working </t>
+  </si>
+  <si>
+    <t xml:space="preserve">window Ihrms desktop </t>
+  </si>
+  <si>
+    <t>task manger not end task the project if it's done auto restart</t>
   </si>
 </sst>
 </file>
@@ -982,7 +1000,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -2885,8 +2903,8 @@
       <c r="E95" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="F95" s="8" t="s">
-        <v>53</v>
+      <c r="F95" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.35">
@@ -2894,7 +2912,7 @@
         <v>46310</v>
       </c>
       <c r="B96" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C96" s="18" t="s">
         <v>146</v>
@@ -2905,7 +2923,67 @@
       <c r="E96" s="19" t="s">
         <v>151</v>
       </c>
-      <c r="F96" s="8" t="s">
+      <c r="F96" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A97" s="2">
+        <v>46311</v>
+      </c>
+      <c r="B97" s="2">
+        <v>46311</v>
+      </c>
+      <c r="C97" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E97" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="F97" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A98" s="2">
+        <v>46311</v>
+      </c>
+      <c r="B98" s="2">
+        <v>46311</v>
+      </c>
+      <c r="C98" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E98" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="F98" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A99" s="2">
+        <v>46311</v>
+      </c>
+      <c r="B99" s="2">
+        <v>46311</v>
+      </c>
+      <c r="C99" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="D99" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E99" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="F99" s="8" t="s">
         <v>53</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement configurable screenshot capture and compression
- Add local configuration for screenshot capture settings.
- Support window-change, interval-based, and combined capture modes.
- Make screenshot capture intervals configurable.
- Prevent duplicate screenshots for the same window.
- Compress screenshots to meet the configured maximum file size.
- Delete screenshots that remain oversized after compression.
- Prevent rejected screenshots from entering the upload queue or database.
- Keep API integration unchanged for future implementation.
- Preserve existing application functionality and Windows/macOS compatibility.
</commit_message>
<xml_diff>
--- a/Monitoring Doc/Project_Task_Tracker (1).xlsx
+++ b/Monitoring Doc/Project_Task_Tracker (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C14CAABD-AF40-4198-ABA9-9B2FB5B39BFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7208B81-0FEB-4E8A-B30F-36883F4099F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="173">
   <si>
     <t>Start Date</t>
   </si>
@@ -512,6 +512,51 @@
   </si>
   <si>
     <t>task manger not end task the project if it's done auto restart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ui window ihrms </t>
+  </si>
+  <si>
+    <t xml:space="preserve">improving  ui and fix the timesheet or addditional task </t>
+  </si>
+  <si>
+    <t>mac implementation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">implement the mac version and restart function on according to windows </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Full name change </t>
+  </si>
+  <si>
+    <t xml:space="preserve">workpulse to ihrms desktop on full project </t>
+  </si>
+  <si>
+    <t xml:space="preserve">change the version 1.1 to 1.0.0 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> version release</t>
+  </si>
+  <si>
+    <t>release the new version on github repo window exe and mac dmg</t>
+  </si>
+  <si>
+    <t>login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alpha bridge attandence or </t>
+  </si>
+  <si>
+    <t xml:space="preserve">send screenshot 100kb to 150kb if then not compress delete in application don’t send this in DB </t>
+  </si>
+  <si>
+    <t>screenshots</t>
+  </si>
+  <si>
+    <t>online take screenshot when window change config</t>
+  </si>
+  <si>
+    <t xml:space="preserve">screenshot time manage config upload in backend /db </t>
   </si>
 </sst>
 </file>
@@ -1000,7 +1045,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F108"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -2166,8 +2211,8 @@
       <c r="E58" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="F58" s="8" t="s">
-        <v>53</v>
+      <c r="F58" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
@@ -2854,13 +2899,13 @@
       <c r="B93" s="2">
         <v>46309</v>
       </c>
-      <c r="C93" s="18" t="s">
+      <c r="C93" s="16" t="s">
         <v>148</v>
       </c>
       <c r="D93" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E93" s="19" t="s">
+      <c r="E93" s="17" t="s">
         <v>149</v>
       </c>
       <c r="F93" s="6" t="s">
@@ -2874,7 +2919,7 @@
       <c r="B94" s="2">
         <v>46310</v>
       </c>
-      <c r="C94" s="18" t="s">
+      <c r="C94" s="16" t="s">
         <v>148</v>
       </c>
       <c r="D94" s="12" t="s">
@@ -2894,13 +2939,13 @@
       <c r="B95" s="2">
         <v>46311</v>
       </c>
-      <c r="C95" s="18" t="s">
+      <c r="C95" s="16" t="s">
         <v>144</v>
       </c>
       <c r="D95" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E95" s="19" t="s">
+      <c r="E95" s="17" t="s">
         <v>142</v>
       </c>
       <c r="F95" s="6" t="s">
@@ -2914,13 +2959,13 @@
       <c r="B96" s="2">
         <v>46311</v>
       </c>
-      <c r="C96" s="18" t="s">
+      <c r="C96" s="16" t="s">
         <v>146</v>
       </c>
       <c r="D96" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E96" s="19" t="s">
+      <c r="E96" s="17" t="s">
         <v>151</v>
       </c>
       <c r="F96" s="6" t="s">
@@ -2934,17 +2979,17 @@
       <c r="B97" s="2">
         <v>46311</v>
       </c>
-      <c r="C97" s="18" t="s">
+      <c r="C97" s="16" t="s">
         <v>152</v>
       </c>
       <c r="D97" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E97" s="19" t="s">
+      <c r="E97" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="F97" s="8" t="s">
-        <v>53</v>
+      <c r="F97" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.35">
@@ -2954,17 +2999,17 @@
       <c r="B98" s="2">
         <v>46311</v>
       </c>
-      <c r="C98" s="18" t="s">
+      <c r="C98" s="16" t="s">
         <v>154</v>
       </c>
       <c r="D98" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E98" s="19" t="s">
+      <c r="E98" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="F98" s="8" t="s">
-        <v>53</v>
+      <c r="F98" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.35">
@@ -2974,16 +3019,196 @@
       <c r="B99" s="2">
         <v>46311</v>
       </c>
-      <c r="C99" s="18" t="s">
+      <c r="C99" s="16" t="s">
         <v>156</v>
       </c>
       <c r="D99" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E99" s="19" t="s">
+      <c r="E99" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="F99" s="8" t="s">
+      <c r="F99" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A100" s="2">
+        <v>46312</v>
+      </c>
+      <c r="B100" s="2">
+        <v>46312</v>
+      </c>
+      <c r="C100" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E100" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="F100" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A101" s="2">
+        <v>46314</v>
+      </c>
+      <c r="B101" s="2">
+        <v>46314</v>
+      </c>
+      <c r="C101" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="D101" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E101" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="F101" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A102" s="2">
+        <v>46316</v>
+      </c>
+      <c r="B102" s="2">
+        <v>46316</v>
+      </c>
+      <c r="C102" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="D102" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E102" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="F102" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A103" s="2">
+        <v>46316</v>
+      </c>
+      <c r="B103" s="2">
+        <v>46316</v>
+      </c>
+      <c r="C103" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="D103" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E103" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="F103" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A104" s="2">
+        <v>46317</v>
+      </c>
+      <c r="B104" s="2">
+        <v>46317</v>
+      </c>
+      <c r="C104" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="D104" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E104" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="F104" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A105" s="2">
+        <v>46318</v>
+      </c>
+      <c r="B105" s="2">
+        <v>46318</v>
+      </c>
+      <c r="C105" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E105" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="F105" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" ht="25" x14ac:dyDescent="0.35">
+      <c r="A106" s="2">
+        <v>46322</v>
+      </c>
+      <c r="B106" s="2">
+        <v>46322</v>
+      </c>
+      <c r="C106" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="D106" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E106" s="19" t="s">
+        <v>169</v>
+      </c>
+      <c r="F106" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A107" s="2">
+        <v>46322</v>
+      </c>
+      <c r="B107" s="2">
+        <v>46322</v>
+      </c>
+      <c r="C107" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="D107" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E107" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="F107" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A108" s="2">
+        <v>46322</v>
+      </c>
+      <c r="B108" s="2">
+        <v>46322</v>
+      </c>
+      <c r="C108" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="D108" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E108" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="F108" s="8" t="s">
         <v>53</v>
       </c>
     </row>

</xml_diff>